<commit_message>
feat: student portfolio v2 — 11 new submissions across W5/W9/W11/W12/W13/W14
- Add Week 5 (Phonology 2) group with 3 entries: 박상언, 박주환, 이환웅
- Add Week 9 (Vowels 1) group with 2 entries: 김지현/이수림/조규현 group project, 이석주
- Append to existing W11: 정유진, 허윤선
- Append to existing W12: 박태훈 (CodePen), 정우재
- Append to existing W13: 오소령
- Append to existing W14: 김의연
- Add platform-codepen CSS class
- Fix stats-box: 11→23 submissions, 8→10 weeks, 5→7 platforms
- Add 9 local student HTML submission files + v2 source xlsx

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/student data/2026-01/26-01 음운론 학생 포트폴리오.xlsx
+++ b/student data/2026-01/26-01 음운론 학생 포트폴리오.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kyunghee\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kyunghee\Desktop\음운론 수업 준비\student data\2026-01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F35888CF-1393-44B9-8670-BA4995F8BC05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B095CB6-5DAA-4091-BBA3-E9DED19FC9BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{D4363A6E-1CAA-4643-95ED-FA195A31C012}"/>
+    <workbookView xWindow="2370" yWindow="1220" windowWidth="7030" windowHeight="11170" xr2:uid="{D4363A6E-1CAA-4643-95ED-FA195A31C012}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>